<commit_message>
Add Day 8 analysis GIF
</commit_message>
<xml_diff>
--- a/Month-1/Day-08/Hungerstation Logistics & Delivery Fleet Dashboard.xlsx
+++ b/Month-1/Day-08/Hungerstation Logistics & Delivery Fleet Dashboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data-Analysis-and-AI-85Days\Month-1\Day-8\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data-Analysis-and-AI-85Days\Month-1\Day-08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089BFF4D-B0FF-46B9-80E9-C20E37233F17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5759392E-966E-48B6-95F9-4CC92F993FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{88D4364E-7EF7-4403-A28E-AC9F1EAAC678}"/>
   </bookViews>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="18" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -514,7 +514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -549,21 +549,26 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -575,37 +580,31 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -619,80 +618,6 @@
           <color indexed="64"/>
         </left>
         <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$⃁-401]\ #,##0.00"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
         <top style="thin">
           <color indexed="64"/>
         </top>
@@ -720,6 +645,22 @@
     <dxf>
       <numFmt numFmtId="164" formatCode="[$⃁-401]\ #,##0.00"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$⃁-401]\ #,##0.00"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -735,6 +676,21 @@
         </bottom>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -758,6 +714,21 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -777,6 +748,21 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -792,6 +778,19 @@
         </bottom>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -820,13 +819,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -843,6 +835,13 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -968,27 +967,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="4"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst>
-              <a:glow rad="63500">
-                <a:schemeClr val="accent1">
-                  <a:satMod val="175000"/>
-                  <a:alpha val="25000"/>
-                </a:schemeClr>
-              </a:glow>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -1052,27 +1031,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="4"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst>
-              <a:glow rad="63500">
-                <a:schemeClr val="accent2">
-                  <a:satMod val="175000"/>
-                  <a:alpha val="25000"/>
-                </a:schemeClr>
-              </a:glow>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -1136,27 +1095,7 @@
           </a:effectLst>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="4"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst>
-              <a:glow rad="63500">
-                <a:schemeClr val="accent3">
-                  <a:satMod val="175000"/>
-                  <a:alpha val="25000"/>
-                </a:schemeClr>
-              </a:glow>
-            </a:effectLst>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -2715,8 +2654,8 @@
       <xdr:row>29</xdr:row>
       <xdr:rowOff>109904</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="5" name="أسم المندوب">
@@ -2739,7 +2678,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -3056,7 +2995,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3147ACA9-1307-4349-8E24-EFF2EDC22A43}" name="PivotTable3" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3147ACA9-1307-4349-8E24-EFF2EDC22A43}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="K14:N30" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField showAll="0"/>
@@ -3279,7 +3218,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{58BA4B2E-7849-4E58-869B-D228FEFE2729}" name="Table1" displayName="Table1" ref="B3:G24" totalsRowCount="1" headerRowDxfId="16" dataDxfId="15" headerRowBorderDxfId="13" tableBorderDxfId="14" totalsRowBorderDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{58BA4B2E-7849-4E58-869B-D228FEFE2729}" name="Table1" displayName="Table1" ref="B3:G24" totalsRowCount="1" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13" totalsRowBorderDxfId="12">
   <autoFilter ref="B3:G23" xr:uid="{58BA4B2E-7849-4E58-869B-D228FEFE2729}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -3292,12 +3231,12 @@
     <sortCondition ref="C3:C23"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{C34EED98-9A92-4FF7-AB37-6ADC9C301B53}" name="رقم المندوب" totalsRowLabel="Total" dataDxfId="11" totalsRowDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{51234773-63CE-47AC-B284-79F8D8152598}" name="أسم المندوب" totalsRowFunction="count" dataDxfId="10" totalsRowDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{9E5135DB-CC42-4C59-BF4F-DFEB65644E35}" name="المدينة" totalsRowFunction="count" dataDxfId="9" totalsRowDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{736F6384-6E94-4C41-A203-667E35CC0424}" name="الطلبات المُسلمة" totalsRowFunction="count" dataDxfId="8" totalsRowDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{A9B3A1FA-75CA-4C5C-83E9-69B6C560E928}" name="رسوم التوصيل" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{A709B46A-E791-4DBE-99AB-9ED8B2B4613E}" name="مصاريف البنزين" totalsRowFunction="custom" dataDxfId="6" totalsRowDxfId="0">
+    <tableColumn id="1" xr3:uid="{C34EED98-9A92-4FF7-AB37-6ADC9C301B53}" name="رقم المندوب" totalsRowLabel="Total" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{51234773-63CE-47AC-B284-79F8D8152598}" name="أسم المندوب" totalsRowFunction="count" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{9E5135DB-CC42-4C59-BF4F-DFEB65644E35}" name="المدينة" totalsRowFunction="count" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{736F6384-6E94-4C41-A203-667E35CC0424}" name="الطلبات المُسلمة" totalsRowFunction="count" dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{A9B3A1FA-75CA-4C5C-83E9-69B6C560E928}" name="رسوم التوصيل" totalsRowFunction="sum" dataDxfId="3" totalsRowDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{A709B46A-E791-4DBE-99AB-9ED8B2B4613E}" name="مصاريف البنزين" totalsRowFunction="custom" dataDxfId="1" totalsRowDxfId="0">
       <totalsRowFormula>SUM(G4:G23)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -3622,7 +3561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9C4DE04-05D7-4D54-A5D1-300078CB69CC}">
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
@@ -3632,46 +3571,46 @@
     <col min="5" max="5" width="17.90625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.7265625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:17">
+      <c r="A1" s="31" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="E1" s="12"/>
-      <c r="F1" s="12"/>
-      <c r="G1" s="12"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
     </row>
-    <row r="2" spans="1:18" ht="14.5" customHeight="1">
-      <c r="A2" s="15"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="19" t="s">
+    <row r="2" spans="1:17" ht="14.5" customHeight="1">
+      <c r="A2" s="31"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
-      <c r="P2" s="20"/>
-      <c r="Q2" s="21"/>
+      <c r="L2" s="23"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="24"/>
     </row>
-    <row r="3" spans="1:18" ht="14.5" customHeight="1">
-      <c r="A3" s="15"/>
+    <row r="3" spans="1:17" ht="14.5" customHeight="1">
+      <c r="A3" s="31"/>
       <c r="B3" s="5" t="s">
         <v>34</v>
       </c>
@@ -3690,17 +3629,17 @@
       <c r="G3" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J3" s="17"/>
+      <c r="J3" s="12"/>
       <c r="K3" s="25"/>
-      <c r="L3" s="23"/>
-      <c r="M3" s="23"/>
-      <c r="N3" s="23"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="23"/>
-      <c r="Q3" s="24"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="27"/>
     </row>
-    <row r="4" spans="1:18" ht="18.5">
-      <c r="A4" s="15"/>
+    <row r="4" spans="1:17" ht="18.5">
+      <c r="A4" s="31"/>
       <c r="B4" s="3">
         <v>106</v>
       </c>
@@ -3719,21 +3658,21 @@
       <c r="G4" s="4">
         <v>30</v>
       </c>
-      <c r="J4" s="18"/>
-      <c r="K4" s="26">
+      <c r="J4" s="13"/>
+      <c r="K4" s="20">
         <v>307</v>
       </c>
-      <c r="L4" s="26"/>
-      <c r="M4" s="27" t="s">
+      <c r="L4" s="20"/>
+      <c r="M4" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28"/>
     </row>
-    <row r="5" spans="1:18" ht="18.5">
-      <c r="A5" s="15"/>
+    <row r="5" spans="1:17" ht="18.5">
+      <c r="A5" s="31"/>
       <c r="B5" s="3">
         <v>101</v>
       </c>
@@ -3752,21 +3691,21 @@
       <c r="G5" s="4">
         <v>45</v>
       </c>
-      <c r="J5" s="18"/>
-      <c r="K5" s="28">
+      <c r="J5" s="13"/>
+      <c r="K5" s="18">
         <v>4605</v>
       </c>
-      <c r="L5" s="28"/>
-      <c r="M5" s="27" t="s">
+      <c r="L5" s="18"/>
+      <c r="M5" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="N5" s="27"/>
-      <c r="O5" s="27"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
+      <c r="N5" s="28"/>
+      <c r="O5" s="28"/>
+      <c r="P5" s="28"/>
+      <c r="Q5" s="28"/>
     </row>
-    <row r="6" spans="1:18" ht="18.5">
-      <c r="A6" s="15"/>
+    <row r="6" spans="1:17" ht="18.5">
+      <c r="A6" s="31"/>
       <c r="B6" s="3">
         <v>117</v>
       </c>
@@ -3785,21 +3724,21 @@
       <c r="G6" s="4">
         <v>60</v>
       </c>
-      <c r="J6" s="18"/>
-      <c r="K6" s="28">
+      <c r="J6" s="13"/>
+      <c r="K6" s="18">
         <v>890</v>
       </c>
-      <c r="L6" s="28"/>
-      <c r="M6" s="27" t="s">
+      <c r="L6" s="18"/>
+      <c r="M6" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-      <c r="Q6" s="27"/>
+      <c r="N6" s="28"/>
+      <c r="O6" s="28"/>
+      <c r="P6" s="28"/>
+      <c r="Q6" s="28"/>
     </row>
-    <row r="7" spans="1:18" ht="18.5">
-      <c r="A7" s="15"/>
+    <row r="7" spans="1:17" ht="18.5">
+      <c r="A7" s="31"/>
       <c r="B7" s="3">
         <v>113</v>
       </c>
@@ -3818,21 +3757,21 @@
       <c r="G7" s="4">
         <v>30</v>
       </c>
-      <c r="J7" s="18"/>
-      <c r="K7" s="29">
+      <c r="J7" s="13"/>
+      <c r="K7" s="19">
         <v>15.35</v>
       </c>
-      <c r="L7" s="29"/>
-      <c r="M7" s="27" t="s">
+      <c r="L7" s="19"/>
+      <c r="M7" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="N7" s="27"/>
-      <c r="O7" s="27"/>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
+      <c r="N7" s="28"/>
+      <c r="O7" s="28"/>
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
     </row>
-    <row r="8" spans="1:18" ht="18.5">
-      <c r="A8" s="15"/>
+    <row r="8" spans="1:17" ht="18.5">
+      <c r="A8" s="31"/>
       <c r="B8" s="3">
         <v>114</v>
       </c>
@@ -3851,21 +3790,21 @@
       <c r="G8" s="4">
         <v>45</v>
       </c>
-      <c r="J8" s="18"/>
-      <c r="K8" s="26">
+      <c r="J8" s="13"/>
+      <c r="K8" s="20">
         <v>44.5</v>
       </c>
-      <c r="L8" s="26"/>
-      <c r="M8" s="27" t="s">
+      <c r="L8" s="20"/>
+      <c r="M8" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="N8" s="27"/>
-      <c r="O8" s="27"/>
-      <c r="P8" s="27"/>
-      <c r="Q8" s="27"/>
+      <c r="N8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
+      <c r="Q8" s="28"/>
     </row>
-    <row r="9" spans="1:18" ht="18.5">
-      <c r="A9" s="15"/>
+    <row r="9" spans="1:17" ht="18.5">
+      <c r="A9" s="31"/>
       <c r="B9" s="3">
         <v>104</v>
       </c>
@@ -3884,21 +3823,21 @@
       <c r="G9" s="4">
         <v>60</v>
       </c>
-      <c r="J9" s="18"/>
-      <c r="K9" s="34">
+      <c r="J9" s="13"/>
+      <c r="K9" s="21">
         <v>20</v>
       </c>
-      <c r="L9" s="26"/>
-      <c r="M9" s="27" t="s">
+      <c r="L9" s="20"/>
+      <c r="M9" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="N9" s="27"/>
-      <c r="O9" s="27"/>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="27"/>
+      <c r="N9" s="28"/>
+      <c r="O9" s="28"/>
+      <c r="P9" s="28"/>
+      <c r="Q9" s="28"/>
     </row>
-    <row r="10" spans="1:18">
-      <c r="A10" s="15"/>
+    <row r="10" spans="1:17">
+      <c r="A10" s="31"/>
       <c r="B10" s="3">
         <v>102</v>
       </c>
@@ -3917,18 +3856,15 @@
       <c r="G10" s="4">
         <v>50</v>
       </c>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="22"/>
-      <c r="P10" s="22"/>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="16"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="14"/>
     </row>
-    <row r="11" spans="1:18">
-      <c r="A11" s="15"/>
+    <row r="11" spans="1:17">
+      <c r="A11" s="31"/>
       <c r="B11" s="3">
         <v>120</v>
       </c>
@@ -3947,16 +3883,9 @@
       <c r="G11" s="4">
         <v>70</v>
       </c>
-      <c r="K11" s="16"/>
-      <c r="L11" s="16"/>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="16"/>
-      <c r="Q11" s="16"/>
     </row>
-    <row r="12" spans="1:18">
-      <c r="A12" s="15"/>
+    <row r="12" spans="1:17">
+      <c r="A12" s="31"/>
       <c r="B12" s="3">
         <v>107</v>
       </c>
@@ -3975,13 +3904,9 @@
       <c r="G12" s="4">
         <v>45</v>
       </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="16"/>
     </row>
-    <row r="13" spans="1:18">
-      <c r="A13" s="15"/>
+    <row r="13" spans="1:17">
+      <c r="A13" s="31"/>
       <c r="B13" s="3">
         <v>103</v>
       </c>
@@ -4000,13 +3925,9 @@
       <c r="G13" s="4">
         <v>35</v>
       </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="16"/>
     </row>
-    <row r="14" spans="1:18">
-      <c r="A14" s="15"/>
+    <row r="14" spans="1:17">
+      <c r="A14" s="31"/>
       <c r="B14" s="3">
         <v>118</v>
       </c>
@@ -4025,7 +3946,7 @@
       <c r="G14" s="4">
         <v>35</v>
       </c>
-      <c r="K14" s="31" t="s">
+      <c r="K14" s="16" t="s">
         <v>50</v>
       </c>
       <c r="L14" t="s">
@@ -4038,8 +3959,8 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:18">
-      <c r="A15" s="15"/>
+    <row r="15" spans="1:17">
+      <c r="A15" s="31"/>
       <c r="B15" s="3">
         <v>111</v>
       </c>
@@ -4058,21 +3979,21 @@
       <c r="G15" s="4">
         <v>40</v>
       </c>
-      <c r="K15" s="32" t="s">
+      <c r="K15" s="17" t="s">
         <v>18</v>
       </c>
       <c r="L15" s="33">
         <v>13</v>
       </c>
-      <c r="M15" s="30">
+      <c r="M15" s="15">
         <v>40</v>
       </c>
-      <c r="N15" s="30">
+      <c r="N15" s="15">
         <v>195</v>
       </c>
     </row>
-    <row r="16" spans="1:18">
-      <c r="A16" s="15"/>
+    <row r="16" spans="1:17">
+      <c r="A16" s="31"/>
       <c r="B16" s="3">
         <v>115</v>
       </c>
@@ -4091,21 +4012,21 @@
       <c r="G16" s="4">
         <v>25</v>
       </c>
-      <c r="K16" s="32" t="s">
+      <c r="K16" s="17" t="s">
         <v>5</v>
       </c>
       <c r="L16" s="33">
         <v>12</v>
       </c>
-      <c r="M16" s="30">
+      <c r="M16" s="15">
         <v>35</v>
       </c>
-      <c r="N16" s="30">
+      <c r="N16" s="15">
         <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="15"/>
+      <c r="A17" s="31"/>
       <c r="B17" s="3">
         <v>109</v>
       </c>
@@ -4124,21 +4045,21 @@
       <c r="G17" s="4">
         <v>35</v>
       </c>
-      <c r="K17" s="32" t="s">
+      <c r="K17" s="17" t="s">
         <v>26</v>
       </c>
       <c r="L17" s="33">
         <v>8</v>
       </c>
-      <c r="M17" s="30">
+      <c r="M17" s="15">
         <v>25</v>
       </c>
-      <c r="N17" s="30">
+      <c r="N17" s="15">
         <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="15"/>
+      <c r="A18" s="31"/>
       <c r="B18" s="3">
         <v>116</v>
       </c>
@@ -4157,21 +4078,21 @@
       <c r="G18" s="4">
         <v>40</v>
       </c>
-      <c r="K18" s="32" t="s">
+      <c r="K18" s="17" t="s">
         <v>3</v>
       </c>
       <c r="L18" s="33">
         <v>43</v>
       </c>
-      <c r="M18" s="30">
+      <c r="M18" s="15">
         <v>125</v>
       </c>
-      <c r="N18" s="30">
+      <c r="N18" s="15">
         <v>645</v>
       </c>
     </row>
     <row r="19" spans="1:14">
-      <c r="A19" s="15"/>
+      <c r="A19" s="31"/>
       <c r="B19" s="3">
         <v>108</v>
       </c>
@@ -4190,21 +4111,21 @@
       <c r="G19" s="4">
         <v>55</v>
       </c>
-      <c r="K19" s="32" t="s">
+      <c r="K19" s="17" t="s">
         <v>24</v>
       </c>
       <c r="L19" s="33">
         <v>15</v>
       </c>
-      <c r="M19" s="30">
+      <c r="M19" s="15">
         <v>45</v>
       </c>
-      <c r="N19" s="30">
+      <c r="N19" s="15">
         <v>225</v>
       </c>
     </row>
     <row r="20" spans="1:14">
-      <c r="A20" s="15"/>
+      <c r="A20" s="31"/>
       <c r="B20" s="3">
         <v>105</v>
       </c>
@@ -4223,21 +4144,21 @@
       <c r="G20" s="4">
         <v>40</v>
       </c>
-      <c r="K20" s="32" t="s">
+      <c r="K20" s="17" t="s">
         <v>30</v>
       </c>
       <c r="L20" s="33">
         <v>21</v>
       </c>
-      <c r="M20" s="30">
+      <c r="M20" s="15">
         <v>60</v>
       </c>
-      <c r="N20" s="30">
+      <c r="N20" s="15">
         <v>315</v>
       </c>
     </row>
     <row r="21" spans="1:14">
-      <c r="A21" s="15"/>
+      <c r="A21" s="31"/>
       <c r="B21" s="3">
         <v>110</v>
       </c>
@@ -4256,21 +4177,21 @@
       <c r="G21" s="4">
         <v>50</v>
       </c>
-      <c r="K21" s="32" t="s">
+      <c r="K21" s="17" t="s">
         <v>16</v>
       </c>
       <c r="L21" s="33">
         <v>17</v>
       </c>
-      <c r="M21" s="30">
+      <c r="M21" s="15">
         <v>50</v>
       </c>
-      <c r="N21" s="30">
+      <c r="N21" s="15">
         <v>255</v>
       </c>
     </row>
     <row r="22" spans="1:14">
-      <c r="A22" s="15"/>
+      <c r="A22" s="31"/>
       <c r="B22" s="3">
         <v>119</v>
       </c>
@@ -4289,21 +4210,21 @@
       <c r="G22" s="4">
         <v>45</v>
       </c>
-      <c r="K22" s="32" t="s">
+      <c r="K22" s="17" t="s">
         <v>8</v>
       </c>
       <c r="L22" s="33">
         <v>14</v>
       </c>
-      <c r="M22" s="30">
+      <c r="M22" s="15">
         <v>40</v>
       </c>
-      <c r="N22" s="30">
+      <c r="N22" s="15">
         <v>210</v>
       </c>
     </row>
     <row r="23" spans="1:14">
-      <c r="A23" s="15"/>
+      <c r="A23" s="31"/>
       <c r="B23" s="8">
         <v>112</v>
       </c>
@@ -4322,16 +4243,16 @@
       <c r="G23" s="11">
         <v>55</v>
       </c>
-      <c r="K23" s="32" t="s">
+      <c r="K23" s="17" t="s">
         <v>11</v>
       </c>
       <c r="L23" s="33">
         <v>16</v>
       </c>
-      <c r="M23" s="30">
+      <c r="M23" s="15">
         <v>45</v>
       </c>
-      <c r="N23" s="30">
+      <c r="N23" s="15">
         <v>240</v>
       </c>
     </row>
@@ -4359,124 +4280,124 @@
         <f>SUM(G4:G23)</f>
         <v>890</v>
       </c>
-      <c r="K24" s="32" t="s">
+      <c r="K24" s="17" t="s">
         <v>28</v>
       </c>
       <c r="L24" s="33">
         <v>14</v>
       </c>
-      <c r="M24" s="30">
+      <c r="M24" s="15">
         <v>40</v>
       </c>
-      <c r="N24" s="30">
+      <c r="N24" s="15">
         <v>210</v>
       </c>
     </row>
     <row r="25" spans="1:14">
-      <c r="K25" s="32" t="s">
+      <c r="K25" s="17" t="s">
         <v>14</v>
       </c>
       <c r="L25" s="33">
         <v>11</v>
       </c>
-      <c r="M25" s="30">
+      <c r="M25" s="15">
         <v>35</v>
       </c>
-      <c r="N25" s="30">
+      <c r="N25" s="15">
         <v>165</v>
       </c>
     </row>
     <row r="26" spans="1:14">
-      <c r="K26" s="32" t="s">
+      <c r="K26" s="17" t="s">
         <v>1</v>
       </c>
       <c r="L26" s="33">
         <v>82</v>
       </c>
-      <c r="M26" s="30">
+      <c r="M26" s="15">
         <v>230</v>
       </c>
-      <c r="N26" s="30">
+      <c r="N26" s="15">
         <v>1230</v>
       </c>
     </row>
     <row r="27" spans="1:14">
-      <c r="K27" s="32" t="s">
+      <c r="K27" s="17" t="s">
         <v>20</v>
       </c>
       <c r="L27" s="33">
         <v>19</v>
       </c>
-      <c r="M27" s="30">
+      <c r="M27" s="15">
         <v>55</v>
       </c>
-      <c r="N27" s="30">
+      <c r="N27" s="15">
         <v>285</v>
       </c>
     </row>
     <row r="28" spans="1:14">
-      <c r="A28" s="14"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="K28" s="32" t="s">
+      <c r="A28" s="32"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="K28" s="17" t="s">
         <v>22</v>
       </c>
       <c r="L28" s="33">
         <v>10</v>
       </c>
-      <c r="M28" s="30">
+      <c r="M28" s="15">
         <v>30</v>
       </c>
-      <c r="N28" s="30">
+      <c r="N28" s="15">
         <v>150</v>
       </c>
     </row>
     <row r="29" spans="1:14">
-      <c r="K29" s="32" t="s">
+      <c r="K29" s="17" t="s">
         <v>32</v>
       </c>
       <c r="L29" s="33">
         <v>12</v>
       </c>
-      <c r="M29" s="30">
+      <c r="M29" s="15">
         <v>35</v>
       </c>
-      <c r="N29" s="30">
+      <c r="N29" s="15">
         <v>180</v>
       </c>
     </row>
     <row r="30" spans="1:14">
-      <c r="K30" s="32" t="s">
+      <c r="K30" s="17" t="s">
         <v>51</v>
       </c>
       <c r="L30" s="33">
         <v>307</v>
       </c>
-      <c r="M30" s="30">
+      <c r="M30" s="15">
         <v>890</v>
       </c>
-      <c r="N30" s="30">
+      <c r="N30" s="15">
         <v>4605</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="M7:Q7"/>
+    <mergeCell ref="M8:Q8"/>
+    <mergeCell ref="M9:Q9"/>
+    <mergeCell ref="B1:G2"/>
+    <mergeCell ref="A1:A23"/>
+    <mergeCell ref="K2:Q3"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="M5:Q5"/>
+    <mergeCell ref="M6:Q6"/>
     <mergeCell ref="K5:L5"/>
     <mergeCell ref="K6:L6"/>
     <mergeCell ref="K7:L7"/>
     <mergeCell ref="K8:L8"/>
     <mergeCell ref="K9:L9"/>
-    <mergeCell ref="K2:Q3"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="M5:Q5"/>
-    <mergeCell ref="M6:Q6"/>
-    <mergeCell ref="M7:Q7"/>
-    <mergeCell ref="M8:Q8"/>
-    <mergeCell ref="M9:Q9"/>
-    <mergeCell ref="B1:G2"/>
-    <mergeCell ref="A1:A23"/>
-    <mergeCell ref="A28:C28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
@@ -4494,21 +4415,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C75CCA8C93D93A43A1AC488E2F0D8821" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1e8fad8455d7b5c89a93d4178a3fc1c9">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d6bf451c-e3aa-4dd1-b5a6-a95183d31bdf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8408199938cbb8869539c7a2b993ecc3" ns3:_="">
     <xsd:import namespace="d6bf451c-e3aa-4dd1-b5a6-a95183d31bdf"/>
@@ -4652,31 +4558,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7090A6C6-DEB4-497C-9A03-DA796E8A5B7D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="d6bf451c-e3aa-4dd1-b5a6-a95183d31bdf"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39F136B9-8709-45A0-B4A2-C966135F8893}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E743430-AB7C-4B0F-9CA5-32165851B708}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4692,4 +4589,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39F136B9-8709-45A0-B4A2-C966135F8893}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7090A6C6-DEB4-497C-9A03-DA796E8A5B7D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="d6bf451c-e3aa-4dd1-b5a6-a95183d31bdf"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>